<commit_message>
#62 Node Design Client BOM Updated Files.
</commit_message>
<xml_diff>
--- a/Deliverable/BOM/eSpark_Ezlo_Voice_Assistant_Node.xlsx
+++ b/Deliverable/BOM/eSpark_Ezlo_Voice_Assistant_Node.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Ezlo-VoiceAssistant\Deliverable\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E77C85AA-0392-4AE6-B590-8A0DE3D7CFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC6E430-4C6A-49DE-80A5-8331B6928E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="418">
   <si>
     <t>Component list</t>
   </si>
@@ -1274,7 +1274,16 @@
     <t>DZ254R-11-05-63</t>
   </si>
   <si>
-    <t>Need Custom Supplier Quote</t>
+    <t xml:space="preserve">Custom Supplier </t>
+  </si>
+  <si>
+    <t>Karen Quote</t>
+  </si>
+  <si>
+    <t>LY68L6400SLIT</t>
+  </si>
+  <si>
+    <t>C261881</t>
   </si>
 </sst>
 </file>
@@ -1286,7 +1295,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1470,14 +1479,6 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1792,7 +1793,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1977,6 +1978,24 @@
     <xf numFmtId="166" fontId="15" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2009,53 +2028,17 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2415,7 +2398,7 @@
     <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.140625" customWidth="1"/>
     <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
@@ -2433,15 +2416,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="68"/>
-      <c r="R1" s="68"/>
-      <c r="S1" s="69"/>
+      <c r="K1" s="74"/>
+      <c r="L1" s="74"/>
+      <c r="M1" s="74"/>
+      <c r="N1" s="74"/>
+      <c r="O1" s="74"/>
+      <c r="P1" s="74"/>
+      <c r="Q1" s="74"/>
+      <c r="R1" s="74"/>
+      <c r="S1" s="75"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2491,7 +2474,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="70"/>
+      <c r="S3" s="76"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2516,7 +2499,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="71"/>
+      <c r="S4" s="77"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2541,7 +2524,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="71"/>
+      <c r="S5" s="77"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2562,7 +2545,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="71"/>
+      <c r="S6" s="77"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2583,7 +2566,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="71"/>
+      <c r="S7" s="77"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2604,7 +2587,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="71"/>
+      <c r="S8" s="77"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -3189,7 +3172,7 @@
       <c r="F19" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="G19" s="80" t="s">
+      <c r="G19" s="68" t="s">
         <v>188</v>
       </c>
       <c r="H19" s="50" t="s">
@@ -3525,7 +3508,7 @@
       <c r="F25" s="50" t="s">
         <v>142</v>
       </c>
-      <c r="G25" s="80" t="s">
+      <c r="G25" s="68" t="s">
         <v>193</v>
       </c>
       <c r="H25" s="50" t="s">
@@ -3749,7 +3732,7 @@
       <c r="F29" s="50" t="s">
         <v>142</v>
       </c>
-      <c r="G29" s="80" t="s">
+      <c r="G29" s="68" t="s">
         <v>197</v>
       </c>
       <c r="H29" s="50" t="s">
@@ -4029,7 +4012,7 @@
       <c r="F34" s="46" t="s">
         <v>153</v>
       </c>
-      <c r="G34" s="81" t="s">
+      <c r="G34" s="69" t="s">
         <v>199</v>
       </c>
       <c r="H34" s="46" t="s">
@@ -4459,53 +4442,63 @@
       <c r="R41" s="64"/>
       <c r="S41" s="52"/>
     </row>
-    <row r="42" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="1"/>
+    <row r="42" spans="1:19" s="87" customFormat="1" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="86"/>
       <c r="B42" s="38">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C42" s="82" t="s">
+      <c r="C42" s="60" t="s">
         <v>398</v>
       </c>
-      <c r="D42" s="83" t="s">
+      <c r="D42" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="E42" s="84" t="s">
+      <c r="E42" s="47" t="s">
         <v>105</v>
       </c>
-      <c r="F42" s="83" t="s">
+      <c r="F42" s="46" t="s">
         <v>311</v>
       </c>
-      <c r="G42" s="83" t="s">
+      <c r="G42" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="H42" s="83" t="s">
+      <c r="H42" s="46" t="s">
         <v>241</v>
       </c>
-      <c r="I42" s="83"/>
-      <c r="J42" s="83"/>
-      <c r="K42" s="83" t="s">
-        <v>313</v>
-      </c>
-      <c r="L42" s="84">
+      <c r="I42" s="84" t="s">
+        <v>313</v>
+      </c>
+      <c r="J42" s="84" t="s">
+        <v>313</v>
+      </c>
+      <c r="K42" s="84" t="s">
+        <v>313</v>
+      </c>
+      <c r="L42" s="85">
         <v>4</v>
       </c>
-      <c r="M42" s="83">
+      <c r="M42" s="46">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N42" s="83"/>
-      <c r="O42" s="85"/>
-      <c r="P42" s="86"/>
-      <c r="Q42" s="86">
+      <c r="N42" s="46">
+        <v>80</v>
+      </c>
+      <c r="O42" s="62" t="s">
+        <v>414</v>
+      </c>
+      <c r="P42" s="53">
+        <v>2.9</v>
+      </c>
+      <c r="Q42" s="53">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>232</v>
       </c>
       <c r="R42" s="65" t="s">
-        <v>414</v>
-      </c>
-      <c r="S42" s="87"/>
+        <v>415</v>
+      </c>
+      <c r="S42" s="70"/>
     </row>
     <row r="43" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
@@ -4525,7 +4518,7 @@
       <c r="F43" s="50" t="s">
         <v>160</v>
       </c>
-      <c r="G43" s="80">
+      <c r="G43" s="68">
         <v>61300211121</v>
       </c>
       <c r="H43" s="50" t="s">
@@ -4581,7 +4574,7 @@
       <c r="F44" s="46" t="s">
         <v>161</v>
       </c>
-      <c r="G44" s="81">
+      <c r="G44" s="69">
         <v>61300611121</v>
       </c>
       <c r="H44" s="46" t="s">
@@ -5368,7 +5361,7 @@
       <c r="F58" s="46" t="s">
         <v>163</v>
       </c>
-      <c r="G58" s="81" t="s">
+      <c r="G58" s="69" t="s">
         <v>211</v>
       </c>
       <c r="H58" s="46" t="s">
@@ -6245,101 +6238,119 @@
       <c r="R73" s="64"/>
       <c r="S73" s="52"/>
     </row>
-    <row r="74" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:19" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="38">
         <f>ROW(B74) - ROW($B$9)</f>
         <v>65</v>
       </c>
-      <c r="C74" s="82" t="s">
+      <c r="C74" s="60" t="s">
         <v>402</v>
       </c>
-      <c r="D74" s="83" t="s">
+      <c r="D74" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="E74" s="84" t="s">
+      <c r="E74" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="F74" s="83" t="s">
+      <c r="F74" s="46" t="s">
         <v>311</v>
       </c>
-      <c r="G74" s="83" t="s">
+      <c r="G74" s="46" t="s">
         <v>177</v>
       </c>
-      <c r="H74" s="83" t="s">
+      <c r="H74" s="46" t="s">
         <v>252</v>
       </c>
-      <c r="I74" s="83"/>
-      <c r="J74" s="83"/>
-      <c r="K74" s="83" t="s">
-        <v>313</v>
-      </c>
-      <c r="L74" s="84">
+      <c r="I74" s="46" t="s">
+        <v>313</v>
+      </c>
+      <c r="J74" s="46" t="s">
+        <v>313</v>
+      </c>
+      <c r="K74" s="46" t="s">
+        <v>313</v>
+      </c>
+      <c r="L74" s="47">
         <v>1</v>
       </c>
-      <c r="M74" s="83">
+      <c r="M74" s="46">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="N74" s="83"/>
-      <c r="O74" s="85"/>
-      <c r="P74" s="86"/>
-      <c r="Q74" s="86">
+      <c r="N74" s="46">
+        <v>11</v>
+      </c>
+      <c r="O74" s="62" t="s">
+        <v>414</v>
+      </c>
+      <c r="P74" s="53">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="Q74" s="53">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="R74" s="92" t="s">
-        <v>414</v>
-      </c>
-      <c r="S74" s="87"/>
-    </row>
-    <row r="75" spans="1:19" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>12.76</v>
+      </c>
+      <c r="R74" s="72" t="s">
+        <v>415</v>
+      </c>
+      <c r="S74" s="70"/>
+    </row>
+    <row r="75" spans="1:19" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="38">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
-      <c r="C75" s="88" t="s">
+      <c r="C75" s="59" t="s">
         <v>402</v>
       </c>
-      <c r="D75" s="79" t="s">
+      <c r="D75" s="50" t="s">
         <v>69</v>
       </c>
-      <c r="E75" s="78" t="s">
+      <c r="E75" s="51" t="s">
         <v>138</v>
       </c>
-      <c r="F75" s="79" t="s">
+      <c r="F75" s="50" t="s">
         <v>169</v>
       </c>
-      <c r="G75" s="79">
+      <c r="G75" s="68">
         <v>4677</v>
       </c>
-      <c r="H75" s="79" t="s">
+      <c r="H75" s="50" t="s">
         <v>253</v>
       </c>
-      <c r="I75" s="79"/>
-      <c r="J75" s="79"/>
-      <c r="K75" s="79" t="s">
-        <v>313</v>
-      </c>
-      <c r="L75" s="78">
+      <c r="I75" s="50" t="s">
+        <v>416</v>
+      </c>
+      <c r="J75" s="50" t="s">
+        <v>417</v>
+      </c>
+      <c r="K75" s="50" t="s">
+        <v>313</v>
+      </c>
+      <c r="L75" s="51">
         <v>1</v>
       </c>
-      <c r="M75" s="79">
+      <c r="M75" s="50">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="N75" s="79"/>
-      <c r="O75" s="89"/>
-      <c r="P75" s="90"/>
-      <c r="Q75" s="90">
+      <c r="N75" s="50">
+        <v>11</v>
+      </c>
+      <c r="O75" s="63" t="s">
+        <v>414</v>
+      </c>
+      <c r="P75" s="54">
+        <v>2.7662</v>
+      </c>
+      <c r="Q75" s="54">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="R75" s="93" t="s">
-        <v>414</v>
-      </c>
-      <c r="S75" s="91"/>
+        <v>30.4282</v>
+      </c>
+      <c r="R75" s="73"/>
+      <c r="S75" s="71"/>
     </row>
     <row r="76" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
@@ -6467,17 +6478,17 @@
       <c r="K78" s="37"/>
       <c r="L78" s="37"/>
       <c r="M78" s="37"/>
-      <c r="N78" s="76" t="s">
+      <c r="N78" s="82" t="s">
         <v>406</v>
       </c>
-      <c r="O78" s="77"/>
-      <c r="P78" s="77"/>
+      <c r="O78" s="83"/>
+      <c r="P78" s="83"/>
       <c r="Q78" s="66">
         <f>SUM(Q10:Q77)</f>
-        <v>189.4359</v>
-      </c>
-      <c r="R78" s="72"/>
-      <c r="S78" s="73"/>
+        <v>464.62409999999994</v>
+      </c>
+      <c r="R78" s="78"/>
+      <c r="S78" s="79"/>
     </row>
     <row r="79" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
@@ -6493,17 +6504,17 @@
       <c r="K79" s="10"/>
       <c r="L79" s="10"/>
       <c r="M79" s="10"/>
-      <c r="N79" s="76" t="s">
+      <c r="N79" s="82" t="s">
         <v>407</v>
       </c>
-      <c r="O79" s="77"/>
-      <c r="P79" s="77"/>
+      <c r="O79" s="83"/>
+      <c r="P79" s="83"/>
       <c r="Q79" s="67">
         <f>Q78/10</f>
-        <v>18.94359</v>
-      </c>
-      <c r="R79" s="74"/>
-      <c r="S79" s="75"/>
+        <v>46.462409999999991</v>
+      </c>
+      <c r="R79" s="80"/>
+      <c r="S79" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>